<commit_message>
Add Framer Motion animations, Stellaris redesign, doctor image upload, interactive calendar, and AI chat interface
</commit_message>
<xml_diff>
--- a/token_usage.xlsx
+++ b/token_usage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT-Project-1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DevProjects\Python\New folder\PH-ITI-W1T1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD695931-DB44-47D7-B370-536631160352}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C53FA8E-0C62-4E28-89A4-C482FE46BDC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{33161382-F3A4-4882-AC9F-7307B57BF6AA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{33161382-F3A4-4882-AC9F-7307B57BF6AA}"/>
   </bookViews>
   <sheets>
     <sheet name="token_usage" sheetId="1" r:id="rId1"/>
@@ -591,9 +591,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -631,7 +631,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -737,7 +737,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -879,7 +879,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -888,17 +888,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A36E89B-E16E-4CD2-9E74-68B337EC9CFA}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -918,7 +918,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>

</xml_diff>